<commit_message>
Update demand planning test cases to use existing table data
- Changed from 'user prepares' to 'user queries/identifies' approach
- Test cases now reference clinical_subject_summary and treatment_groups tables
- Steps reflect real testing workflow: query tables to find conditions, then test results
- More realistic for database-driven testing scenarios
</commit_message>
<xml_diff>
--- a/Demand_Planning_Module_Test_Cases.xlsx
+++ b/Demand_Planning_Module_Test_Cases.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="83">
   <si>
     <t>Test Scenario ID</t>
   </si>
@@ -61,15 +61,15 @@
     <t>Generate a medicine demand forecast for active patients based on their treatment schedules</t>
   </si>
   <si>
-    <t>Step 1: User places curated Subject Summary file and Treatment Mapping file in the designated input folders.
+    <t>Step 1: User verifies that clinical_subject_summary table and treatment_groups table contain active patient data.
 Step 2: User initiates the demand planning process.
-Step 3: User opens the demand forecast output file.
+Step 3: User opens the demand forecast output table.
 Step 4: User verifies that projected visits are calculated for all active patients.
 Step 5: User verifies that visit dates span approximately 365 days into the future.
-Step 6: User verifies that medicine quantities are calculated correctly based on visit frequency and dispensing rules.</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary + Treatment Mapping files</t>
+Step 6: User verifies that medicine quantities are calculated correctly based on visit frequency and dispensing rules from treatment_groups table.</t>
+  </si>
+  <si>
+    <t>clinical_subject_summary + treatment_groups tables</t>
   </si>
   <si>
     <t>50 active patients with standard treatment protocols</t>
@@ -87,18 +87,18 @@
     <t>Validation that only active patients are included in demand forecast</t>
   </si>
   <si>
-    <t>Step 1: User prepares Subject Summary file containing 100 patients with various statuses: 60 Active/Randomized, 20 Screen Failed, 10 Treatment Discontinued, 10 Pre-Screened Failed.
-Step 2: User initiates the demand planning process.
-Step 3: User opens the demand forecast output.
-Step 4: User counts unique patients in the output.
-Step 5: User verifies that only 60 patients appear (Active/Randomized status).
+    <t>Step 1: User queries clinical_subject_summary table and identifies patients with various statuses (Active/Randomized, Screen Failed, Treatment Discontinued, Pre-Screened Failed).
+Step 2: User counts patients with active statuses vs excluded statuses.
+Step 3: User initiates the demand planning process.
+Step 4: User opens the demand forecast output table and counts unique patients.
+Step 5: User verifies that only patients with active statuses appear in the forecast output.
 Step 6: User verifies that Screen Failed, Treatment Discontinued, and Pre-Screened Failed patients do NOT appear in the output.</t>
   </si>
   <si>
-    <t>Curated Subject Summary with mixed patient statuses</t>
-  </si>
-  <si>
-    <t>100 patients with 40% excluded statuses</t>
+    <t>clinical_subject_summary table with mixed patient statuses</t>
+  </si>
+  <si>
+    <t>Patients with various status values in subject_status column</t>
   </si>
   <si>
     <t>DP-MATCH-01</t>
@@ -113,18 +113,18 @@
     <t>Validation that patients are matched to country-specific treatment protocols when available</t>
   </si>
   <si>
-    <t>Step 1: User prepares Treatment Mapping file with country-specific protocols: Protocol A for USA, Protocol A for Canada, Protocol A for Germany (same study, different countries).
-Step 2: User prepares Subject Summary with patients from USA, Canada, and Germany all on Protocol A.
+    <t>Step 1: User queries treatment_groups table and identifies protocols with country-specific mappings (e.g., same study_protocol for USA, Canada, Germany with different visit schedules).
+Step 2: User queries clinical_subject_summary table and identifies patients from these countries on the same study protocol.
 Step 3: User initiates the demand planning process.
-Step 4: User opens the demand forecast output.
+Step 4: User opens the demand forecast output table.
 Step 5: User filters patients by country and verifies each country's patients received their country-specific treatment protocol (different visit schedules or drug quantities).
 Step 6: User verifies that USA patients do NOT receive Canada protocol and vice versa.</t>
   </si>
   <si>
-    <t>Curated Subject Summary + Treatment Mapping with country variations</t>
-  </si>
-  <si>
-    <t>Patients from 3 countries on same study protocol</t>
+    <t>clinical_subject_summary + treatment_groups tables with country variations</t>
+  </si>
+  <si>
+    <t>Patients from multiple countries with country-specific treatment mappings</t>
   </si>
   <si>
     <t>DP-MATCH-02</t>
@@ -136,18 +136,18 @@
     <t>Validation that patients receive generic treatment protocol when no country-specific mapping exists</t>
   </si>
   <si>
-    <t>Step 1: User prepares Treatment Mapping file with country-specific protocols for USA and Canada, plus one generic protocol (country field blank) for Protocol B.
-Step 2: User prepares Subject Summary with patients from USA, Canada, and Japan all on Protocol B.
+    <t>Step 1: User queries treatment_groups table and identifies protocols with both country-specific and generic mappings (country field blank/null).
+Step 2: User queries clinical_subject_summary table and identifies patients from countries with and without specific mappings.
 Step 3: User initiates the demand planning process.
-Step 4: User opens the demand forecast output.
-Step 5: User verifies that USA and Canada patients matched to their country-specific Protocol B mappings.
-Step 6: User verifies that Japan patients (no country-specific mapping) matched to the generic Protocol B mapping.</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary + Treatment Mapping with mixed country/generic protocols</t>
-  </si>
-  <si>
-    <t>Patients from 3 countries with different mapping availability</t>
+Step 4: User opens the demand forecast output table.
+Step 5: User verifies that patients from countries with specific mappings matched to their country-specific protocols.
+Step 6: User verifies that patients from countries without specific mappings matched to the generic protocol.</t>
+  </si>
+  <si>
+    <t>clinical_subject_summary + treatment_groups tables with mixed country/generic protocols</t>
+  </si>
+  <si>
+    <t>Patients from countries with varying mapping availability</t>
   </si>
   <si>
     <t>DP-VISIT-01</t>
@@ -162,15 +162,12 @@
     <t>Validation that remaining visits in patient's current cycle are projected correctly</t>
   </si>
   <si>
-    <t>Step 1: User prepares Subject Summary with patient whose last visit was Cycle 5 Day 1 on 2025-01-01.
-Step 2: User prepares Treatment Mapping with visit schedule: Days 1, 8, 15 (28-day cycles).
-Step 3: User initiates the demand planning process (assume today is 2025-01-05).
-Step 4: User opens the demand forecast output and filters to this patient.
-Step 5: User verifies that 2 remaining visits are projected for current Cycle 5: Day 8 (2025-01-08) and Day 15 (2025-01-15).
-Step 6: User verifies that Cycle 6 visits begin after Cycle 5 Day 15.</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary with specific last visit + Treatment Mapping</t>
+    <t>Step 1: User queries clinical_subject_summary table and identifies a patient whose last_study_visit_recorded shows mid-cycle status (e.g., Cycle 5 Day 1).
+Step 2: User queries treatment_groups table to find this patient's visit schedule (e.g., Days 1, 8, 15 with 28-day cycles).
+Step 3: User initiates the demand planning process.
+Step 4: User opens the demand forecast output table and filters to this patient.
+Step 5: User verifies that remaining visits in the current cycle are projected (e.g., Day 8 and Day 15 for Cycle 5).
+Step 6: User verifies that next cycle visits begin after current cycle completes.</t>
   </si>
   <si>
     <t>Single patient mid-cycle with known visit schedule</t>
@@ -185,18 +182,15 @@
     <t>Validation that future complete cycles are projected correctly within 365-day window</t>
   </si>
   <si>
-    <t>Step 1: User prepares Subject Summary with patient whose last visit was Cycle 1 Day 15 on 2025-01-15 (cycle complete).
-Step 2: User prepares Treatment Mapping with visit schedule: Days 1, 8, 15 (28-day cycles), no max cycles defined.
-Step 3: User initiates the demand planning process (assume today is 2025-01-20).
-Step 4: User opens the demand forecast output and filters to this patient.
-Step 5: User verifies that approximately 13 future cycles are projected (365 days ÷ 28 days per cycle).
-Step 6: User verifies that Cycle 2 Day 1 starts on 2025-01-29 (28 days after Cycle 1 Day 1).</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary with completed cycle + Treatment Mapping</t>
-  </si>
-  <si>
-    <t>Single patient ready for next cycle</t>
+    <t>Step 1: User queries clinical_subject_summary table and identifies a patient whose last_study_visit_recorded shows completed cycle (e.g., Cycle 1 Day 15 where Day 15 is the last visit day).
+Step 2: User queries treatment_groups table to confirm this patient's cycle length and visit schedule.
+Step 3: User initiates the demand planning process.
+Step 4: User opens the demand forecast output table and filters to this patient.
+Step 5: User counts the number of future cycles projected and verifies it aligns with 365-day projection window.
+Step 6: User verifies that next cycle Day 1 date is calculated correctly based on dispensing_frequency_days from treatment_groups table.</t>
+  </si>
+  <si>
+    <t>Single patient with completed cycle ready for future cycles</t>
   </si>
   <si>
     <t>DP-VISIT-03</t>
@@ -208,18 +202,15 @@
     <t>Validation that visits beyond 365 days from today are NOT included in forecast</t>
   </si>
   <si>
-    <t>Step 1: User prepares Subject Summary with patient on Cycle 1 Day 1 dated 2025-01-01.
-Step 2: User prepares Treatment Mapping with 28-day cycles, Days 1, 15 visit schedule, no max cycles.
-Step 3: User initiates the demand planning process (assume today is 2025-01-15).
-Step 4: User opens the demand forecast output and filters to this patient.
+    <t>Step 1: User queries clinical_subject_summary table and identifies a patient with early cycle visit (e.g., Cycle 1 Day 1) that could potentially generate many future cycles.
+Step 2: User queries treatment_groups table to confirm this patient has no max_cycles constraint (or high max_cycles value).
+Step 3: User initiates the demand planning process and notes today's date.
+Step 4: User opens the demand forecast output table and filters to this patient.
 Step 5: User identifies the last projected visit date in the output.
-Step 6: User verifies that no visits are projected beyond 2026-01-15 (365 days from today 2025-01-15).</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary + Treatment Mapping with long projection potential</t>
-  </si>
-  <si>
-    <t>Single patient with unlimited cycles</t>
+Step 6: User verifies that no visits are projected beyond 365 days from today's date.</t>
+  </si>
+  <si>
+    <t>Single patient with unlimited or high max_cycles</t>
   </si>
   <si>
     <t>DP-VISIT-04</t>
@@ -228,21 +219,18 @@
     <t>Max Cycles Constraint Enforcement</t>
   </si>
   <si>
-    <t>Validation that patients with max cycles defined do not exceed the cycle limit</t>
-  </si>
-  <si>
-    <t>Step 1: User prepares Subject Summary with patient on Cycle 8 Day 15 (last recorded visit).
-Step 2: User prepares Treatment Mapping with max_cycles = 10, 28-day cycles, Days 1, 15 visit schedule.
+    <t>Validation that patients with max_cycles defined do not exceed the cycle limit</t>
+  </si>
+  <si>
+    <t>Step 1: User queries treatment_groups table and identifies a protocol with max_cycles constraint defined (e.g., max_cycles = 10).
+Step 2: User queries clinical_subject_summary table and identifies a patient on this protocol who is near the max cycle limit (e.g., Cycle 8 Day 15).
 Step 3: User initiates the demand planning process.
-Step 4: User opens the demand forecast output and filters to this patient.
-Step 5: User verifies that visits are projected only through Cycle 10 (maximum allowed).
-Step 6: User verifies that NO Cycle 11 visits appear, even if within 365-day window.</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary + Treatment Mapping with max_cycles defined</t>
-  </si>
-  <si>
-    <t>Patient near max cycles limit</t>
+Step 4: User opens the demand forecast output table and filters to this patient.
+Step 5: User verifies that visits are projected only through the max_cycles limit (e.g., Cycle 10).
+Step 6: User verifies that NO visits appear beyond the max_cycles limit, even if within 365-day window.</t>
+  </si>
+  <si>
+    <t>Patient near max_cycles limit with max_cycles defined in treatment_groups</t>
   </si>
   <si>
     <t>DP-TREAT-04</t>
@@ -257,18 +245,15 @@
     <t>Validation that crossover patients are labeled correctly in projected visits</t>
   </si>
   <si>
-    <t>Step 1: User prepares Subject Summary with patient whose last visit is "Crossover Cycle 2 Day 1".
-Step 2: User prepares Treatment Mapping for crossover protocol (visit Days 1, 15, 28-day cycles).
+    <t>Step 1: User queries clinical_subject_summary table and identifies a patient whose last_study_visit_recorded contains "Crossover" (e.g., "Crossover Cycle 2 Day 1").
+Step 2: User queries treatment_groups table to confirm this patient's crossover protocol visit schedule.
 Step 3: User initiates the demand planning process.
-Step 4: User opens the demand forecast output and filters to this patient.
-Step 5: User verifies that all projected visits include "Crossover" prefix (e.g. "Crossover Cycle 3 Day 1").
+Step 4: User opens the demand forecast output table and filters to this patient.
+Step 5: User verifies that all projected visits in predicted_study_visit column include "Crossover" prefix (e.g., "Crossover Cycle 3 Day 1").
 Step 6: User verifies that cycle numbering continues sequentially from last recorded cycle.</t>
   </si>
   <si>
-    <t>Curated Subject Summary with crossover patient + Treatment Mapping</t>
-  </si>
-  <si>
-    <t>Single crossover patient</t>
+    <t>Single crossover patient identified in clinical_subject_summary</t>
   </si>
   <si>
     <t>DP-MULTI-01</t>
@@ -283,18 +268,15 @@
     <t>Validation that patients receiving multiple study drugs have separate forecasts per drug</t>
   </si>
   <si>
-    <t>Step 1: User prepares Treatment Mapping with Protocol A defining: study_drug_dispensed = "Drug-A" AND additional_study_drug_dispensed = "Drug-B".
-Step 2: User prepares Subject Summary with 1 patient on Protocol A, Cycle 5 Day 1 last visit.
+    <t>Step 1: User queries treatment_groups table and identifies a protocol where both study_drug_dispensed AND additional_study_drug_dispensed are populated (e.g., Drug-A and Drug-B).
+Step 2: User queries clinical_subject_summary table and identifies a patient assigned to this multi-drug protocol.
 Step 3: User initiates the demand planning process.
-Step 4: User opens the demand forecast output and filters to this patient (subject_number).
-Step 5: User verifies that patient has TWO sets of projected visits: one for Drug-A and one for Drug-B.
-Step 6: User verifies that both drugs show identical visit schedules but are listed as separate drugs.</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary + Treatment Mapping with multiple drugs</t>
-  </si>
-  <si>
-    <t>Single patient on multi-drug protocol</t>
+Step 4: User opens the demand forecast output table and filters to this patient (subject_number).
+Step 5: User verifies that patient has TWO sets of projected visits: one for Drug-A and one for Drug-B in the drug_dispensed column.
+Step 6: User verifies that both drugs show identical visit schedules but are listed as separate drug entries.</t>
+  </si>
+  <si>
+    <t>Single patient on multi-drug protocol with both drug columns populated</t>
   </si>
   <si>
     <t>DP-ERR-01</t>
@@ -309,18 +291,15 @@
     <t>Validation of handling when patient's treatment protocol is not in the mapping file</t>
   </si>
   <si>
-    <t>Step 1: User prepares Subject Summary with patient on "Protocol-XYZ" that does NOT exist in Treatment Mapping file.
+    <t>Step 1: User queries clinical_subject_summary table and identifies a patient with a study_protocol, randomized_treatment, tpc, or subject_status combination that does NOT exist in treatment_groups table.
 Step 2: User initiates the demand planning process.
 Step 3: User checks processing logs or error reports.
-Step 4: User verifies that system provides clear message indicating unmapped protocol for patient.
-Step 5: User verifies that other patients with valid mappings are still processed successfully.
-Step 6: User verifies that unmapped patient does NOT appear in demand forecast output.</t>
-  </si>
-  <si>
-    <t>Curated Subject Summary with unmapped protocol + Treatment Mapping</t>
-  </si>
-  <si>
-    <t>1 patient with non-existent protocol, 9 patients with valid protocols</t>
+Step 4: User verifies that system provides clear message indicating unmapped protocol for this patient.
+Step 5: User verifies that other patients with valid mappings in treatment_groups are still processed successfully.
+Step 6: User verifies that unmapped patient does NOT appear in demand forecast output table.</t>
+  </si>
+  <si>
+    <t>Patient with combination not mapped in treatment_groups table</t>
   </si>
   <si>
     <t>DP-OUT-01</t>
@@ -336,16 +315,13 @@
   </si>
   <si>
     <t>Step 1: User reviews expected output column list: study_name, parent_depot, site_id, subject_number, subject_status, subject_country, randomized_treatment, tpc, drug_dispensed, dispensing_quantity, predicted_study_visit, cycle, day, predicted_next_visit_date, processed_timestamp.
-Step 2: User processes standard dataset through demand planning.
-Step 3: User opens the demand forecast output file.
-Step 4: User verifies that all 15 expected columns are present.
+Step 2: User initiates demand planning process using clinical_subject_summary and treatment_groups tables.
+Step 3: User opens the demand forecast output table.
+Step 4: User verifies that all 15 expected columns are present in the output table.
 Step 5: User verifies no unexpected columns are included.</t>
   </si>
   <si>
-    <t>Curated Subject Summary + Treatment Mapping</t>
-  </si>
-  <si>
-    <t>Standard dataset with 20 patients</t>
+    <t>Standard patient dataset from clinical tables</t>
   </si>
 </sst>
 </file>
@@ -885,10 +861,10 @@
         <v>42</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>44</v>
       </c>
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
@@ -897,25 +873,25 @@
     </row>
     <row r="7" spans="1:11" ht="150" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="E7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="F7" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>50</v>
       </c>
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
@@ -924,25 +900,25 @@
     </row>
     <row r="8" spans="1:11" ht="150" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C8" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="F8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>56</v>
       </c>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
@@ -951,25 +927,25 @@
     </row>
     <row r="9" spans="1:11" ht="150" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>39</v>
       </c>
       <c r="C9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -978,25 +954,25 @@
     </row>
     <row r="10" spans="1:11" ht="150" customHeight="1">
       <c r="A10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="F10" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="F10" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="G10" s="2" t="s">
-        <v>69</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -1005,25 +981,25 @@
     </row>
     <row r="11" spans="1:11" ht="150" customHeight="1">
       <c r="A11" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="2" t="s">
         <v>70</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F11" s="2" t="s">
-        <v>75</v>
-      </c>
-      <c r="G11" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -1032,25 +1008,25 @@
     </row>
     <row r="12" spans="1:11" ht="150" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1059,25 +1035,25 @@
     </row>
     <row r="13" spans="1:11" ht="150" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>89</v>
+        <v>16</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>

</xml_diff>